<commit_message>
Meter paises nuevos y mas cosas
</commit_message>
<xml_diff>
--- a/datos/paises.xlsx
+++ b/datos/paises.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manue\OneDrive\Desktop\Juegos\Road to Gold\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D7C4C63-D57F-4660-9431-28683C6A5E13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6DC156-90F7-4C7A-8528-9799C2C43D56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0C12F03E-F4F1-4B58-AEF9-00A818977629}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="73">
   <si>
     <t>id</t>
   </si>
@@ -246,6 +246,18 @@
   </si>
   <si>
     <t>México</t>
+  </si>
+  <si>
+    <t>ARG</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>TPE</t>
+  </si>
+  <si>
+    <t>Taipei</t>
   </si>
 </sst>
 </file>
@@ -617,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{259D404A-F656-47E9-B6EB-214B2E007FEA}">
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
@@ -705,7 +717,7 @@
         <v>5</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F2">
         <v>5</v>
@@ -776,7 +788,7 @@
         <v>9</v>
       </c>
       <c r="E3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3">
         <v>8</v>
@@ -847,7 +859,7 @@
         <v>6</v>
       </c>
       <c r="E4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F4">
         <v>8</v>
@@ -918,7 +930,7 @@
         <v>6</v>
       </c>
       <c r="E5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5">
         <v>5</v>
@@ -990,7 +1002,7 @@
         <v>5</v>
       </c>
       <c r="E6">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F6">
         <v>9</v>
@@ -1278,7 +1290,7 @@
         <v>5</v>
       </c>
       <c r="E10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10">
         <v>6</v>
@@ -1350,7 +1362,7 @@
         <v>2</v>
       </c>
       <c r="E11">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F11">
         <v>8</v>
@@ -1422,7 +1434,7 @@
         <v>7</v>
       </c>
       <c r="E12">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12">
         <v>8</v>
@@ -1782,7 +1794,7 @@
         <v>2</v>
       </c>
       <c r="E17">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17">
         <v>2</v>
@@ -1854,7 +1866,7 @@
         <v>6</v>
       </c>
       <c r="E18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F18">
         <v>4</v>
@@ -2067,7 +2079,7 @@
         <v>3</v>
       </c>
       <c r="E21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F21">
         <v>7</v>
@@ -2121,6 +2133,148 @@
         <v>28</v>
       </c>
       <c r="W21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22">
+        <v>2</v>
+      </c>
+      <c r="H22">
+        <v>4</v>
+      </c>
+      <c r="I22">
+        <v>3</v>
+      </c>
+      <c r="J22">
+        <v>3</v>
+      </c>
+      <c r="K22">
+        <v>5</v>
+      </c>
+      <c r="L22">
+        <v>3</v>
+      </c>
+      <c r="M22">
+        <v>7</v>
+      </c>
+      <c r="N22">
+        <v>5</v>
+      </c>
+      <c r="O22">
+        <v>1</v>
+      </c>
+      <c r="P22">
+        <v>3</v>
+      </c>
+      <c r="Q22">
+        <v>6</v>
+      </c>
+      <c r="R22">
+        <v>6</v>
+      </c>
+      <c r="S22">
+        <v>1</v>
+      </c>
+      <c r="T22">
+        <v>1</v>
+      </c>
+      <c r="U22">
+        <v>0</v>
+      </c>
+      <c r="V22" t="s">
+        <v>28</v>
+      </c>
+      <c r="W22" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" t="s">
+        <v>72</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>4</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>6</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
+      </c>
+      <c r="J23">
+        <v>1</v>
+      </c>
+      <c r="K23">
+        <v>4</v>
+      </c>
+      <c r="L23">
+        <v>4</v>
+      </c>
+      <c r="M23">
+        <v>0</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>3</v>
+      </c>
+      <c r="S23">
+        <v>1</v>
+      </c>
+      <c r="T23">
+        <v>6</v>
+      </c>
+      <c r="U23">
+        <v>8</v>
+      </c>
+      <c r="V23" t="s">
+        <v>40</v>
+      </c>
+      <c r="W23" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Meter fiyi, nueva zelanda y récords de partida rápida
</commit_message>
<xml_diff>
--- a/datos/paises.xlsx
+++ b/datos/paises.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manue\OneDrive\Desktop\Juegos\Road to Gold\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BCA9004-9113-46F4-882C-92CA80F65684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37846D37-C822-406E-9136-04EBD1951DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0C12F03E-F4F1-4B58-AEF9-00A818977629}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="81">
   <si>
     <t>id</t>
   </si>
@@ -270,6 +270,18 @@
   </si>
   <si>
     <t>Austria</t>
+  </si>
+  <si>
+    <t>Fiji</t>
+  </si>
+  <si>
+    <t>FIJ</t>
+  </si>
+  <si>
+    <t>NZL</t>
+  </si>
+  <si>
+    <t>Nueva Zelanda</t>
   </si>
 </sst>
 </file>
@@ -641,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{259D404A-F656-47E9-B6EB-214B2E007FEA}">
-  <dimension ref="A1:Y24"/>
+  <dimension ref="A1:Y26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="21" width="11.42578125" customWidth="1"/>
@@ -2508,6 +2520,160 @@
         <v>3</v>
       </c>
     </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>0</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
+      <c r="T25">
+        <v>0</v>
+      </c>
+      <c r="U25">
+        <v>0</v>
+      </c>
+      <c r="V25">
+        <v>10</v>
+      </c>
+      <c r="W25">
+        <v>0</v>
+      </c>
+      <c r="X25" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26">
+        <v>4</v>
+      </c>
+      <c r="E26">
+        <v>4</v>
+      </c>
+      <c r="F26">
+        <v>2</v>
+      </c>
+      <c r="G26">
+        <v>9</v>
+      </c>
+      <c r="H26">
+        <v>3</v>
+      </c>
+      <c r="I26">
+        <v>8</v>
+      </c>
+      <c r="J26">
+        <v>6</v>
+      </c>
+      <c r="K26">
+        <v>1</v>
+      </c>
+      <c r="L26">
+        <v>3</v>
+      </c>
+      <c r="M26">
+        <v>4</v>
+      </c>
+      <c r="N26">
+        <v>1</v>
+      </c>
+      <c r="O26">
+        <v>1</v>
+      </c>
+      <c r="P26">
+        <v>0</v>
+      </c>
+      <c r="Q26">
+        <v>0</v>
+      </c>
+      <c r="R26">
+        <v>1</v>
+      </c>
+      <c r="S26">
+        <v>0</v>
+      </c>
+      <c r="T26">
+        <v>0</v>
+      </c>
+      <c r="U26">
+        <v>0</v>
+      </c>
+      <c r="V26">
+        <v>10</v>
+      </c>
+      <c r="W26">
+        <v>0</v>
+      </c>
+      <c r="X26" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>